<commit_message>
fix URL, clean code
</commit_message>
<xml_diff>
--- a/src/test/resources/PurchaseFormTestData.xlsx
+++ b/src/test/resources/PurchaseFormTestData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="85">
   <si>
     <t>testId</t>
   </si>
@@ -542,7 +542,7 @@
         <v>41</v>
       </c>
       <c r="Y3" t="s" s="0">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>59</v>
       </c>
       <c r="Y4" t="s" s="0">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">

</xml_diff>